<commit_message>
add new files for program import
</commit_message>
<xml_diff>
--- a/1_Stoichiometry_generator/Results.xlsx
+++ b/1_Stoichiometry_generator/Results.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmitry.bublikov\Downloads\cpp-test-anion\st_32\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmitry.bublikov\Desktop\Desktop\nacl\NaCl-superstructure-simulator\1_Stoichiometry_generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA9B96D3-CE9D-44C5-B5FF-1EDA551B9980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FBF7EC-472F-412B-9621-FA30BF3EBCF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
   <si>
     <t>Components (cations/anions)</t>
   </si>
@@ -56,6 +55,9 @@
   </si>
   <si>
     <t>New in CF108 (CF108-CF32)</t>
+  </si>
+  <si>
+    <t>no data</t>
   </si>
 </sst>
 </file>
@@ -441,7 +443,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -483,6 +485,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -805,11 +813,10 @@
       <c r="C2" s="16">
         <v>1.0416666666666667E-4</v>
       </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="26">
-        <f>D2-B2</f>
-        <v>-8452591</v>
-      </c>
+      <c r="D2" s="34" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="26"/>
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -822,11 +829,10 @@
       <c r="C3" s="14">
         <v>2.8935185185185184E-4</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="27">
-        <f>D3-B3</f>
-        <v>-32861324</v>
-      </c>
+      <c r="D3" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="27"/>
       <c r="F3" s="4"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -839,11 +845,10 @@
       <c r="C4" s="12">
         <v>2.6620370370370372E-4</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="27">
-        <f t="shared" ref="E4:E34" si="0">D4-B4</f>
-        <v>-41515514</v>
-      </c>
+      <c r="D4" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="27"/>
       <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -860,7 +865,7 @@
         <v>50144015603</v>
       </c>
       <c r="E5" s="27">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E4:E34" si="0">D5-B5</f>
         <v>50122201599</v>
       </c>
       <c r="F5" s="22">

</xml_diff>

<commit_message>
add new moduadd new modules, fix modules and readme
</commit_message>
<xml_diff>
--- a/1_Stoichiometry_generator/Results.xlsx
+++ b/1_Stoichiometry_generator/Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmitry.bublikov\Desktop\Desktop\nacl\NaCl-superstructure-simulator\1_Stoichiometry_generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FBF7EC-472F-412B-9621-FA30BF3EBCF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AC19614-F0D7-44F4-8DD6-13E63590BFB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>Components (cations/anions)</t>
   </si>
@@ -779,7 +779,7 @@
     <col min="2" max="2" width="19.90625" customWidth="1"/>
     <col min="3" max="3" width="10.7265625" customWidth="1"/>
     <col min="4" max="4" width="20.90625" customWidth="1"/>
-    <col min="5" max="5" width="23.36328125" customWidth="1"/>
+    <col min="5" max="5" width="23.453125" customWidth="1"/>
     <col min="6" max="6" width="11.7265625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -845,11 +845,16 @@
       <c r="C4" s="12">
         <v>2.6620370370370372E-4</v>
       </c>
-      <c r="D4" s="35" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="27"/>
-      <c r="F4" s="4"/>
+      <c r="D4" s="30">
+        <v>393037764859</v>
+      </c>
+      <c r="E4" s="30">
+        <f t="shared" ref="E4:E34" si="0">D4-B4</f>
+        <v>392996249345</v>
+      </c>
+      <c r="F4" s="22">
+        <v>16.774756944444444</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="10">
@@ -865,7 +870,7 @@
         <v>50144015603</v>
       </c>
       <c r="E5" s="27">
-        <f t="shared" ref="E4:E34" si="0">D5-B5</f>
+        <f t="shared" si="0"/>
         <v>50122201599</v>
       </c>
       <c r="F5" s="22">
@@ -1467,11 +1472,11 @@
       </c>
       <c r="D34" s="29">
         <f>SUM(D2:D33)</f>
-        <v>621438236283</v>
+        <v>1014476001142</v>
       </c>
       <c r="E34" s="29">
         <f t="shared" si="0"/>
-        <v>621260759130</v>
+        <v>1014298523989</v>
       </c>
     </row>
   </sheetData>

</xml_diff>